<commit_message>
DEV: MPJ_15565 - ProjExpenseGeneralJournalLineEntityTemplate fix
git-tfs-id: [https://dev.azure.com/METCASHDevOps]$/Metcash D365 FO Implementation/Trunk/Main;C1426
</commit_message>
<xml_diff>
--- a/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METProjExpenseGeneralJournalLineEntityTemplate.xlsx
+++ b/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METProjExpenseGeneralJournalLineEntityTemplate.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin35b84abf9c\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin10196d7258\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -143,8 +143,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -230,7 +230,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -240,13 +240,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -307,7 +307,28 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <fill>
@@ -364,27 +385,6 @@
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -400,54 +400,54 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A11:X12" insertRow="1" totalsRowShown="0" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A11:X12" insertRow="1" totalsRowShown="0" dataDxfId="18">
   <autoFilter ref="A11:X12"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Date" dataDxfId="17"/>
     <tableColumn id="2" name="Voucher" dataDxfId="16"/>
-    <tableColumn id="3" name="Account type" dataDxfId="15"/>
-    <tableColumn id="4" name="Non-ledger account" dataDxfId="14"/>
-    <tableColumn id="5" name="Main account" dataDxfId="13"/>
-    <tableColumn id="6" name="Financial dimensions" dataDxfId="12"/>
-    <tableColumn id="7" name="Description" dataDxfId="11"/>
-    <tableColumn id="8" name="Debit" dataDxfId="30"/>
-    <tableColumn id="9" name="Credit" dataDxfId="29"/>
-    <tableColumn id="10" name="Offset account type" dataDxfId="10"/>
-    <tableColumn id="11" name="Offset Non-ledger account" dataDxfId="9"/>
-    <tableColumn id="12" name="Offset account" dataDxfId="8"/>
-    <tableColumn id="13" name="Offset financial dimensions" dataDxfId="7"/>
-    <tableColumn id="14" name="Offset transaction text" dataDxfId="6"/>
-    <tableColumn id="15" name="Currency" dataDxfId="5"/>
-    <tableColumn id="16" name="Quantity" dataDxfId="28"/>
-    <tableColumn id="17" name="Category" dataDxfId="4"/>
-    <tableColumn id="18" name="Sales currency" dataDxfId="3"/>
-    <tableColumn id="19" name="Sales price" dataDxfId="27"/>
-    <tableColumn id="20" name="Line property" dataDxfId="2"/>
-    <tableColumn id="21" name="Line number" dataDxfId="26"/>
-    <tableColumn id="22" name="Company" dataDxfId="1"/>
-    <tableColumn id="23" name="Exchange rate" dataDxfId="25"/>
-    <tableColumn id="24" name="Offset company" dataDxfId="0"/>
+    <tableColumn id="3" name="Company" dataDxfId="15"/>
+    <tableColumn id="4" name="Account type" dataDxfId="14"/>
+    <tableColumn id="5" name="Non-ledger account" dataDxfId="13"/>
+    <tableColumn id="6" name="Main account" dataDxfId="12"/>
+    <tableColumn id="7" name="Financial dimensions" dataDxfId="11"/>
+    <tableColumn id="8" name="Description" dataDxfId="10"/>
+    <tableColumn id="9" name="Debit" dataDxfId="24"/>
+    <tableColumn id="10" name="Credit" dataDxfId="23"/>
+    <tableColumn id="11" name="Offset company" dataDxfId="9"/>
+    <tableColumn id="12" name="Offset account type" dataDxfId="8"/>
+    <tableColumn id="13" name="Offset Non-ledger account" dataDxfId="7"/>
+    <tableColumn id="14" name="Offset account" dataDxfId="6"/>
+    <tableColumn id="15" name="Offset financial dimensions" dataDxfId="5"/>
+    <tableColumn id="16" name="Offset transaction text" dataDxfId="4"/>
+    <tableColumn id="17" name="Currency" dataDxfId="3"/>
+    <tableColumn id="18" name="Quantity" dataDxfId="22"/>
+    <tableColumn id="19" name="Category" dataDxfId="2"/>
+    <tableColumn id="20" name="Sales currency" dataDxfId="1"/>
+    <tableColumn id="21" name="Sales price" dataDxfId="21"/>
+    <tableColumn id="22" name="Line property" dataDxfId="0"/>
+    <tableColumn id="23" name="Line number" dataDxfId="20"/>
+    <tableColumn id="24" name="Exchange rate" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <autoFilter ref="A2:B5"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="22"/>
-    <tableColumn id="2" name="Column2" dataDxfId="21"/>
+    <tableColumn id="1" name="Column1" dataDxfId="29"/>
+    <tableColumn id="2" name="Column2" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="D2:D3"/>
   <tableColumns count="1">
-    <tableColumn id="1" name="Column1" dataDxfId="18"/>
+    <tableColumn id="1" name="Column1" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -716,7 +716,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="525" row="4">
+  <wetp:taskpane dockstate="right" visibility="1" width="437" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -727,8 +727,8 @@
   <we:reference id="WA104379629" version="1.3.0.0" store="en-US" storeType="OMEX"/>
   <we:alternateReferences/>
   <we:properties>
-    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev673ef33fbd249d24ddevaos.cloudax.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:true,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1561340370799&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;VoucherDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Voucher&quot;,&quot;LabelId&quot;:&quot;@SYS12371&quot;,&quot;Name&quot;:&quot;Voucher&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Main account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityMainAccount&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Financial dimensions&quot;,&quot;LabelId&quot;:&quot;@SYS138491&quot;,&quot;Name&quot;:&quot;DimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerOffsetAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset account&quot;,&quot;LabelId&quot;:&quot;@SYS11162&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset financial dimensions&quot;,&quot;LabelId&quot;:&quot;@Proj:OffsetFinancialDimensions&quot;,&quot;Name&quot;:&quot;OffsetDefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset transaction text&quot;,&quot;LabelId&quot;:&quot;@SYS24282&quot;,&quot;Name&quot;:&quot;OffsetTransactionText&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Quantity&quot;,&quot;LabelId&quot;:&quot;@SYS14578&quot;,&quot;Name&quot;:&quot;Quantity&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Category&quot;,&quot;LabelId&quot;:&quot;@Proj:Category&quot;,&quot;Name&quot;:&quot;ProjectCategory&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales currency&quot;,&quot;LabelId&quot;:&quot;@SYS56480&quot;,&quot;Name&quot;:&quot;ProjectSalesCurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales price&quot;,&quot;LabelId&quot;:&quot;@SYS5755&quot;,&quot;Name&quot;:&quot;ProjectSalesPrice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line property&quot;,&quot;LabelId&quot;:&quot;@SYS50026&quot;,&quot;Name&quot;:&quot;ProjectLineProperty&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;dataAreaId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Exchange rate&quot;,&quot;LabelId&quot;:&quot;@SYS4955&quot;,&quot;Name&quot;:&quot;ExchangeRate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561187605443&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;},{&quot;Id&quot;:&quot;label-binding-1561187689068&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;},{&quot;Id&quot;:&quot;label-binding-1561187700349&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;},{&quot;Id&quot;:&quot;label-binding-1561187712566&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1561187611697&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187691970&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187702847&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187714846&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561339164024&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;label-binding-1561339226221&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;label-binding-1561339327326&quot;,&quot;Label&quot;:&quot;Totals&quot;,&quot;LabelId&quot;:&quot;@SYS13865&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]}},{&quot;PublicName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]},&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2017-04-06T22:02:44.134Z&quot;,&quot;DocumentId&quot;:&quot;18953a8c-81f6-478e-bca9-9dbabcb2610c&quot;,&quot;GenerationActivityId&quot;:&quot;8CDC58C8-FE6E-40C3-AC6D-AEE77F547D6C&quot;}"/>
     <we:property name="Features" value="{&quot;LogDomEvents&quot;:false,&quot;LogTelemetry&quot;:true}"/>
+    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev20dcaba4bf23405e0devaos.cloudax.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:true,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1561340370799&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;VoucherDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Voucher&quot;,&quot;LabelId&quot;:&quot;@SYS12371&quot;,&quot;Name&quot;:&quot;Voucher&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;dataAreaId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Main account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityMainAccount&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Financial dimensions&quot;,&quot;LabelId&quot;:&quot;@SYS138491&quot;,&quot;Name&quot;:&quot;DimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerOffsetAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset account&quot;,&quot;LabelId&quot;:&quot;@SYS11162&quot;,&quot;Name&quot;:&quot;OffsetAccountDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset financial dimensions&quot;,&quot;LabelId&quot;:&quot;@Proj:OffsetFinancialDimensions&quot;,&quot;Name&quot;:&quot;OffsetDefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset transaction text&quot;,&quot;LabelId&quot;:&quot;@SYS24282&quot;,&quot;Name&quot;:&quot;OffsetTransactionText&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Quantity&quot;,&quot;LabelId&quot;:&quot;@SYS14578&quot;,&quot;Name&quot;:&quot;Quantity&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Category&quot;,&quot;LabelId&quot;:&quot;@Proj:Category&quot;,&quot;Name&quot;:&quot;ProjectCategory&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales currency&quot;,&quot;LabelId&quot;:&quot;@SYS56480&quot;,&quot;Name&quot;:&quot;ProjectSalesCurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales price&quot;,&quot;LabelId&quot;:&quot;@SYS5755&quot;,&quot;Name&quot;:&quot;ProjectSalesPrice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line property&quot;,&quot;LabelId&quot;:&quot;@SYS50026&quot;,&quot;Name&quot;:&quot;ProjectLineProperty&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Exchange rate&quot;,&quot;LabelId&quot;:&quot;@SYS4955&quot;,&quot;Name&quot;:&quot;ExchangeRate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561187605443&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;},{&quot;Id&quot;:&quot;label-binding-1561187689068&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;},{&quot;Id&quot;:&quot;label-binding-1561187700349&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;},{&quot;Id&quot;:&quot;label-binding-1561187712566&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1561187611697&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187691970&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187702847&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187714846&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561339164024&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;label-binding-1561339226221&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;label-binding-1561339327326&quot;,&quot;Label&quot;:&quot;Totals&quot;,&quot;LabelId&quot;:&quot;@SYS13865&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]}},{&quot;PublicName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]},&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2017-04-06T22:02:44.134Z&quot;,&quot;DocumentId&quot;:&quot;18953a8c-81f6-478e-bca9-9dbabcb2610c&quot;,&quot;GenerationActivityId&quot;:&quot;15470A14-A6CB-4D2F-B1BE-4A0832942879&quot;}"/>
   </we:properties>
   <we:bindings>
     <we:binding id="DataCacheKey" type="table" appref="{13626F68-6484-44FA-BEC8-165B23378132}"/>
@@ -753,42 +753,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="25.1796875" customWidth="1"/>
-    <col min="5" max="5" width="19.1796875" customWidth="1"/>
-    <col min="6" max="6" width="26.26953125" customWidth="1"/>
-    <col min="7" max="7" width="18.54296875" customWidth="1"/>
-    <col min="8" max="9" width="13.26953125" customWidth="1"/>
-    <col min="10" max="10" width="25.54296875" customWidth="1"/>
-    <col min="11" max="11" width="34.453125" customWidth="1"/>
-    <col min="12" max="12" width="19.54296875" customWidth="1"/>
-    <col min="13" max="13" width="34.453125" customWidth="1"/>
-    <col min="14" max="14" width="29.1796875" customWidth="1"/>
-    <col min="15" max="15" width="14.54296875" customWidth="1"/>
-    <col min="16" max="16" width="14.26953125" customWidth="1"/>
-    <col min="17" max="17" width="14.453125" customWidth="1"/>
-    <col min="18" max="18" width="19.81640625" customWidth="1"/>
-    <col min="19" max="19" width="16.453125" customWidth="1"/>
-    <col min="20" max="20" width="17.81640625" customWidth="1"/>
-    <col min="21" max="21" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.21875" customWidth="1"/>
+    <col min="6" max="6" width="26.21875" customWidth="1"/>
+    <col min="7" max="7" width="18.5546875" customWidth="1"/>
+    <col min="8" max="9" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="25.5546875" customWidth="1"/>
+    <col min="11" max="11" width="34.44140625" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" customWidth="1"/>
+    <col min="13" max="13" width="34.44140625" customWidth="1"/>
+    <col min="14" max="14" width="29.21875" customWidth="1"/>
+    <col min="15" max="15" width="14.5546875" customWidth="1"/>
+    <col min="16" max="16" width="33.21875" customWidth="1"/>
+    <col min="17" max="17" width="14.44140625" customWidth="1"/>
+    <col min="18" max="18" width="19.77734375" customWidth="1"/>
+    <col min="19" max="19" width="16.44140625" customWidth="1"/>
+    <col min="20" max="20" width="17.77734375" customWidth="1"/>
+    <col min="21" max="21" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -797,7 +797,7 @@
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -806,7 +806,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -815,7 +815,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:24" ht="21" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:24" ht="21" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -824,7 +824,7 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="F8" s="5" t="s">
         <v>8</v>
       </c>
@@ -832,20 +832,20 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="E9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F9" s="6">
+        <f>SUM(Table1[Description])</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
         <f>SUM(Table1[Debit])</f>
         <v>0</v>
       </c>
-      <c r="G9" s="6">
-        <f>SUM(Table1[Credit])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -853,73 +853,73 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
         <v>7</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>30</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>28</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>26</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>3</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>8</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>9</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
+        <v>35</v>
+      </c>
+      <c r="L11" t="s">
         <v>10</v>
       </c>
-      <c r="K11" t="s">
+      <c r="M11" t="s">
         <v>31</v>
       </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>11</v>
       </c>
-      <c r="M11" t="s">
+      <c r="O11" t="s">
         <v>27</v>
       </c>
-      <c r="N11" t="s">
+      <c r="P11" t="s">
         <v>12</v>
       </c>
-      <c r="O11" t="s">
+      <c r="Q11" t="s">
         <v>13</v>
       </c>
-      <c r="P11" t="s">
+      <c r="R11" t="s">
         <v>14</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="S11" t="s">
         <v>15</v>
       </c>
-      <c r="R11" t="s">
+      <c r="T11" t="s">
         <v>16</v>
       </c>
-      <c r="S11" t="s">
+      <c r="U11" t="s">
         <v>17</v>
       </c>
-      <c r="T11" t="s">
+      <c r="V11" t="s">
         <v>18</v>
       </c>
-      <c r="U11" t="s">
+      <c r="W11" t="s">
         <v>25</v>
       </c>
-      <c r="V11" t="s">
-        <v>33</v>
-      </c>
-      <c r="W11" t="s">
+      <c r="X11" t="s">
         <v>34</v>
       </c>
-      <c r="X11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -927,23 +927,23 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="11"/>
+      <c r="H12" s="2"/>
       <c r="I12" s="11"/>
-      <c r="J12" s="2"/>
+      <c r="J12" s="11"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-      <c r="P12" s="11"/>
+      <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="2"/>
       <c r="T12" s="2"/>
       <c r="U12" s="11"/>
       <c r="V12" s="2"/>
       <c r="W12" s="11"/>
-      <c r="X12" s="2"/>
+      <c r="X12" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1005,20 +1005,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11" style="8" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" style="8"/>
+    <col min="3" max="3" width="9.21875" style="8"/>
     <col min="4" max="4" width="11" style="8" customWidth="1"/>
-    <col min="5" max="16384" width="9.1796875" style="8"/>
+    <col min="5" max="16384" width="9.21875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>23</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Dev : MPJ_15565 Excel template Fix
git-tfs-id: [https://dev.azure.com/METCASHDevOps]$/Metcash D365 FO Implementation/Trunk/Main;C1510
</commit_message>
<xml_diff>
--- a/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METProjExpenseGeneralJournalLineEntityTemplate.xlsx
+++ b/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METProjExpenseGeneralJournalLineEntityTemplate.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin10196d7258\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin35b84abf9c\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Project Expense Journal</t>
   </si>
@@ -129,13 +129,16 @@
     <t>&lt;no-data&gt;</t>
   </si>
   <si>
-    <t>Company</t>
-  </si>
-  <si>
     <t>Exchange rate</t>
   </si>
   <si>
     <t>Offset company</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Company2</t>
   </si>
 </sst>
 </file>
@@ -143,8 +146,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -230,7 +233,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -240,13 +243,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -254,60 +257,63 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+  <dxfs count="33">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -400,54 +406,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A11:X12" insertRow="1" totalsRowShown="0" dataDxfId="18">
-  <autoFilter ref="A11:X12"/>
-  <tableColumns count="24">
-    <tableColumn id="1" name="Date" dataDxfId="17"/>
-    <tableColumn id="2" name="Voucher" dataDxfId="16"/>
-    <tableColumn id="3" name="Company" dataDxfId="15"/>
-    <tableColumn id="4" name="Account type" dataDxfId="14"/>
-    <tableColumn id="5" name="Non-ledger account" dataDxfId="13"/>
-    <tableColumn id="6" name="Main account" dataDxfId="12"/>
-    <tableColumn id="7" name="Financial dimensions" dataDxfId="11"/>
-    <tableColumn id="8" name="Description" dataDxfId="10"/>
-    <tableColumn id="9" name="Debit" dataDxfId="24"/>
-    <tableColumn id="10" name="Credit" dataDxfId="23"/>
-    <tableColumn id="11" name="Offset company" dataDxfId="9"/>
-    <tableColumn id="12" name="Offset account type" dataDxfId="8"/>
-    <tableColumn id="13" name="Offset Non-ledger account" dataDxfId="7"/>
-    <tableColumn id="14" name="Offset account" dataDxfId="6"/>
-    <tableColumn id="15" name="Offset financial dimensions" dataDxfId="5"/>
-    <tableColumn id="16" name="Offset transaction text" dataDxfId="4"/>
-    <tableColumn id="17" name="Currency" dataDxfId="3"/>
-    <tableColumn id="18" name="Quantity" dataDxfId="22"/>
-    <tableColumn id="19" name="Category" dataDxfId="2"/>
-    <tableColumn id="20" name="Sales currency" dataDxfId="1"/>
-    <tableColumn id="21" name="Sales price" dataDxfId="21"/>
-    <tableColumn id="22" name="Line property" dataDxfId="0"/>
-    <tableColumn id="23" name="Line number" dataDxfId="20"/>
-    <tableColumn id="24" name="Exchange rate" dataDxfId="19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A11:Y12" insertRow="1" totalsRowShown="0" dataDxfId="19">
+  <autoFilter ref="A11:Y12"/>
+  <tableColumns count="25">
+    <tableColumn id="1" name="Date" dataDxfId="18"/>
+    <tableColumn id="2" name="Voucher" dataDxfId="17"/>
+    <tableColumn id="3" name="Company2" dataDxfId="16"/>
+    <tableColumn id="4" name="Account" dataDxfId="15"/>
+    <tableColumn id="5" name="Account type" dataDxfId="14"/>
+    <tableColumn id="6" name="Non-ledger account" dataDxfId="13"/>
+    <tableColumn id="7" name="Main account" dataDxfId="12"/>
+    <tableColumn id="8" name="Financial dimensions" dataDxfId="11"/>
+    <tableColumn id="9" name="Description" dataDxfId="10"/>
+    <tableColumn id="10" name="Debit" dataDxfId="25"/>
+    <tableColumn id="11" name="Credit" dataDxfId="24"/>
+    <tableColumn id="12" name="Offset company" dataDxfId="9"/>
+    <tableColumn id="13" name="Offset account type" dataDxfId="8"/>
+    <tableColumn id="14" name="Offset Non-ledger account" dataDxfId="7"/>
+    <tableColumn id="15" name="Offset account" dataDxfId="6"/>
+    <tableColumn id="16" name="Offset financial dimensions" dataDxfId="5"/>
+    <tableColumn id="17" name="Offset transaction text" dataDxfId="4"/>
+    <tableColumn id="18" name="Currency" dataDxfId="3"/>
+    <tableColumn id="19" name="Quantity" dataDxfId="23"/>
+    <tableColumn id="20" name="Category" dataDxfId="2"/>
+    <tableColumn id="21" name="Sales currency" dataDxfId="1"/>
+    <tableColumn id="22" name="Sales price" dataDxfId="22"/>
+    <tableColumn id="23" name="Line property" dataDxfId="0"/>
+    <tableColumn id="24" name="Line number" dataDxfId="21"/>
+    <tableColumn id="25" name="Exchange rate" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A2:B5"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="29"/>
-    <tableColumn id="2" name="Column2" dataDxfId="28"/>
+    <tableColumn id="1" name="Column1" dataDxfId="30"/>
+    <tableColumn id="2" name="Column2" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="D2:D3"/>
   <tableColumns count="1">
-    <tableColumn id="1" name="Column1" dataDxfId="25"/>
+    <tableColumn id="1" name="Column1" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -716,7 +723,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="437" row="1">
+  <wetp:taskpane dockstate="right" visibility="1" width="350" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -727,8 +734,8 @@
   <we:reference id="WA104379629" version="1.3.0.0" store="en-US" storeType="OMEX"/>
   <we:alternateReferences/>
   <we:properties>
+    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev673ef33fbd249d24ddevaos.cloudax.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:true,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1561340370799&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;VoucherDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Voucher&quot;,&quot;LabelId&quot;:&quot;@SYS12371&quot;,&quot;Name&quot;:&quot;Voucher&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company2&quot;,&quot;Name&quot;:&quot;AccountCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account&quot;,&quot;LabelId&quot;:&quot;@SYS24500&quot;,&quot;Name&quot;:&quot;AccountDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Main account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityMainAccount&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Financial dimensions&quot;,&quot;LabelId&quot;:&quot;@SYS138491&quot;,&quot;Name&quot;:&quot;DimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerOffsetAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset account&quot;,&quot;LabelId&quot;:&quot;@SYS11162&quot;,&quot;Name&quot;:&quot;OffsetAccountDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset financial dimensions&quot;,&quot;LabelId&quot;:&quot;@Proj:OffsetFinancialDimensions&quot;,&quot;Name&quot;:&quot;OffsetDefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset transaction text&quot;,&quot;LabelId&quot;:&quot;@SYS24282&quot;,&quot;Name&quot;:&quot;OffsetTransactionText&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Quantity&quot;,&quot;LabelId&quot;:&quot;@SYS14578&quot;,&quot;Name&quot;:&quot;Quantity&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Category&quot;,&quot;LabelId&quot;:&quot;@Proj:Category&quot;,&quot;Name&quot;:&quot;ProjectCategory&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales currency&quot;,&quot;LabelId&quot;:&quot;@SYS56480&quot;,&quot;Name&quot;:&quot;ProjectSalesCurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales price&quot;,&quot;LabelId&quot;:&quot;@SYS5755&quot;,&quot;Name&quot;:&quot;ProjectSalesPrice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line property&quot;,&quot;LabelId&quot;:&quot;@SYS50026&quot;,&quot;Name&quot;:&quot;ProjectLineProperty&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Exchange rate&quot;,&quot;LabelId&quot;:&quot;@SYS4955&quot;,&quot;Name&quot;:&quot;ExchangeRate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561187605443&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;},{&quot;Id&quot;:&quot;label-binding-1561187689068&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;},{&quot;Id&quot;:&quot;label-binding-1561187700349&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;},{&quot;Id&quot;:&quot;label-binding-1561187712566&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1561187611697&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187691970&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187702847&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187714846&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561339164024&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;label-binding-1561339226221&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;label-binding-1561339327326&quot;,&quot;Label&quot;:&quot;Totals&quot;,&quot;LabelId&quot;:&quot;@SYS13865&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]}},{&quot;PublicName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]},&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2017-04-06T22:02:44.134Z&quot;,&quot;DocumentId&quot;:&quot;18953a8c-81f6-478e-bca9-9dbabcb2610c&quot;,&quot;GenerationActivityId&quot;:&quot;80A88DCE-15B8-4D19-B840-7FE12F9F2FDE&quot;}"/>
     <we:property name="Features" value="{&quot;LogDomEvents&quot;:false,&quot;LogTelemetry&quot;:true}"/>
-    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev20dcaba4bf23405e0devaos.cloudax.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:true,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1561340370799&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;VoucherDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Voucher&quot;,&quot;LabelId&quot;:&quot;@SYS12371&quot;,&quot;Name&quot;:&quot;Voucher&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;dataAreaId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Main account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityMainAccount&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Financial dimensions&quot;,&quot;LabelId&quot;:&quot;@SYS138491&quot;,&quot;Name&quot;:&quot;DimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityNonLedgerOffsetAccount&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;ProjExpenseJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset account&quot;,&quot;LabelId&quot;:&quot;@SYS11162&quot;,&quot;Name&quot;:&quot;OffsetAccountDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset financial dimensions&quot;,&quot;LabelId&quot;:&quot;@Proj:OffsetFinancialDimensions&quot;,&quot;Name&quot;:&quot;OffsetDefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset transaction text&quot;,&quot;LabelId&quot;:&quot;@SYS24282&quot;,&quot;Name&quot;:&quot;OffsetTransactionText&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Quantity&quot;,&quot;LabelId&quot;:&quot;@SYS14578&quot;,&quot;Name&quot;:&quot;Quantity&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Category&quot;,&quot;LabelId&quot;:&quot;@Proj:Category&quot;,&quot;Name&quot;:&quot;ProjectCategory&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales currency&quot;,&quot;LabelId&quot;:&quot;@SYS56480&quot;,&quot;Name&quot;:&quot;ProjectSalesCurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Sales price&quot;,&quot;LabelId&quot;:&quot;@SYS5755&quot;,&quot;Name&quot;:&quot;ProjectSalesPrice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line property&quot;,&quot;LabelId&quot;:&quot;@SYS50026&quot;,&quot;Name&quot;:&quot;ProjectLineProperty&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Exchange rate&quot;,&quot;LabelId&quot;:&quot;@SYS4955&quot;,&quot;Name&quot;:&quot;ExchangeRate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561187605443&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;},{&quot;Id&quot;:&quot;label-binding-1561187689068&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;},{&quot;Id&quot;:&quot;label-binding-1561187700349&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;},{&quot;Id&quot;:&quot;label-binding-1561187712566&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1561187611697&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187691970&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;JournalNameId&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187702847&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1561187714846&quot;,&quot;EntityName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1561339164024&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;label-binding-1561339226221&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;label-binding-1561339327326&quot;,&quot;Label&quot;:&quot;Totals&quot;,&quot;LabelId&quot;:&quot;@SYS13865&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;ExpenseJournalHeader&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]}},{&quot;PublicName&quot;:&quot;ExpenseJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;ussi&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00001&quot;}]},&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2017-04-06T22:02:44.134Z&quot;,&quot;DocumentId&quot;:&quot;18953a8c-81f6-478e-bca9-9dbabcb2610c&quot;,&quot;GenerationActivityId&quot;:&quot;15470A14-A6CB-4D2F-B1BE-4A0832942879&quot;}"/>
   </we:properties>
   <we:bindings>
     <we:binding id="DataCacheKey" type="table" appref="{13626F68-6484-44FA-BEC8-165B23378132}"/>
@@ -752,43 +759,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Y12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.21875" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="25.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.21875" customWidth="1"/>
-    <col min="6" max="6" width="26.21875" customWidth="1"/>
-    <col min="7" max="7" width="18.5546875" customWidth="1"/>
-    <col min="8" max="9" width="13.21875" customWidth="1"/>
-    <col min="10" max="10" width="25.5546875" customWidth="1"/>
-    <col min="11" max="11" width="34.44140625" customWidth="1"/>
-    <col min="12" max="12" width="19.5546875" customWidth="1"/>
-    <col min="13" max="13" width="34.44140625" customWidth="1"/>
-    <col min="14" max="14" width="29.21875" customWidth="1"/>
-    <col min="15" max="15" width="14.5546875" customWidth="1"/>
-    <col min="16" max="16" width="33.21875" customWidth="1"/>
-    <col min="17" max="17" width="14.44140625" customWidth="1"/>
-    <col min="18" max="18" width="19.77734375" customWidth="1"/>
-    <col min="19" max="19" width="16.44140625" customWidth="1"/>
-    <col min="20" max="20" width="17.77734375" customWidth="1"/>
-    <col min="21" max="21" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" customWidth="1"/>
+    <col min="8" max="9" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" customWidth="1"/>
+    <col min="11" max="11" width="34.42578125" customWidth="1"/>
+    <col min="12" max="12" width="19.5703125" customWidth="1"/>
+    <col min="13" max="13" width="34.42578125" customWidth="1"/>
+    <col min="14" max="14" width="29.28515625" customWidth="1"/>
+    <col min="15" max="15" width="14.5703125" customWidth="1"/>
+    <col min="16" max="16" width="33.28515625" customWidth="1"/>
+    <col min="17" max="17" width="14.42578125" customWidth="1"/>
+    <col min="18" max="18" width="19.7109375" customWidth="1"/>
+    <col min="19" max="19" width="16.42578125" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" customWidth="1"/>
+    <col min="21" max="21" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -797,7 +806,7 @@
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -806,7 +815,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -815,7 +824,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:24" ht="21" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -824,7 +833,7 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="F8" s="5" t="s">
         <v>8</v>
       </c>
@@ -832,20 +841,20 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="E9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F9" s="6">
+        <f>SUM(Table1[Financial dimensions])</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
         <f>SUM(Table1[Description])</f>
         <v>0</v>
       </c>
-      <c r="G9" s="6">
-        <f>SUM(Table1[Debit])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -853,73 +862,76 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J11" t="s">
+        <v>8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>9</v>
+      </c>
+      <c r="L11" t="s">
+        <v>34</v>
+      </c>
+      <c r="M11" t="s">
+        <v>10</v>
+      </c>
+      <c r="N11" t="s">
+        <v>31</v>
+      </c>
+      <c r="O11" t="s">
+        <v>11</v>
+      </c>
+      <c r="P11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>12</v>
+      </c>
+      <c r="R11" t="s">
+        <v>13</v>
+      </c>
+      <c r="S11" t="s">
+        <v>14</v>
+      </c>
+      <c r="T11" t="s">
+        <v>15</v>
+      </c>
+      <c r="U11" t="s">
+        <v>16</v>
+      </c>
+      <c r="V11" t="s">
+        <v>17</v>
+      </c>
+      <c r="W11" t="s">
+        <v>18</v>
+      </c>
+      <c r="X11" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y11" t="s">
         <v>33</v>
       </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" t="s">
-        <v>3</v>
-      </c>
-      <c r="I11" t="s">
-        <v>8</v>
-      </c>
-      <c r="J11" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" t="s">
-        <v>35</v>
-      </c>
-      <c r="L11" t="s">
-        <v>10</v>
-      </c>
-      <c r="M11" t="s">
-        <v>31</v>
-      </c>
-      <c r="N11" t="s">
-        <v>11</v>
-      </c>
-      <c r="O11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P11" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>13</v>
-      </c>
-      <c r="R11" t="s">
-        <v>14</v>
-      </c>
-      <c r="S11" t="s">
-        <v>15</v>
-      </c>
-      <c r="T11" t="s">
-        <v>16</v>
-      </c>
-      <c r="U11" t="s">
-        <v>17</v>
-      </c>
-      <c r="V11" t="s">
-        <v>18</v>
-      </c>
-      <c r="W11" t="s">
-        <v>25</v>
-      </c>
-      <c r="X11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -928,22 +940,23 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="11"/>
+      <c r="I12" s="2"/>
       <c r="J12" s="11"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="11"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="11"/>
       <c r="T12" s="2"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="2"/>
-      <c r="W12" s="11"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="11"/>
+      <c r="W12" s="2"/>
       <c r="X12" s="11"/>
+      <c r="Y12" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1005,20 +1018,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11" style="8" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" style="8"/>
+    <col min="3" max="3" width="9.28515625" style="8"/>
     <col min="4" max="4" width="11" style="8" customWidth="1"/>
-    <col min="5" max="16384" width="9.21875" style="8"/>
+    <col min="5" max="16384" width="9.28515625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
@@ -1029,7 +1042,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>23</v>
       </c>
@@ -1037,7 +1050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
@@ -1045,7 +1058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>24</v>
       </c>

</xml_diff>